<commit_message>
agregamos palabras que más se repiten en cada mall
</commit_message>
<xml_diff>
--- a/sandbox/tablas_locales_CC/Ejemplo_correspondencia_recreo_calles.xlsx
+++ b/sandbox/tablas_locales_CC/Ejemplo_correspondencia_recreo_calles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atiscodesa-my.sharepoint.com/personal/ruben_freire_centrohub_co/Documents/Escritorio/Proyectos/CENTROS COMERCIALES/sandbox/tablas_locales_CC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{A0A6E139-C61D-4FE5-9EEC-A2E607BB718F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D3F041C-4B47-46F6-B50C-A5A0479BFD65}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{A0A6E139-C61D-4FE5-9EEC-A2E607BB718F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C3A89D4-3A6A-4BBB-9E28-B7863F085056}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="384" windowWidth="23016" windowHeight="12216" xr2:uid="{B20A79E2-87F7-4978-9B48-C89280278B27}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{B20A79E2-87F7-4978-9B48-C89280278B27}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>centro_comercial</t>
   </si>
@@ -75,6 +75,45 @@
   </si>
   <si>
     <t>LA MAGDALENA</t>
+  </si>
+  <si>
+    <t>MALL DEL SOL</t>
+  </si>
+  <si>
+    <t>GUAYAS</t>
+  </si>
+  <si>
+    <t>GUAYAQUIL</t>
+  </si>
+  <si>
+    <t>TARQUI</t>
+  </si>
+  <si>
+    <t>marengo</t>
+  </si>
+  <si>
+    <t>tanca</t>
+  </si>
+  <si>
+    <t>juan</t>
+  </si>
+  <si>
+    <t>joaquin</t>
+  </si>
+  <si>
+    <t>orratia</t>
+  </si>
+  <si>
+    <t>gonzales</t>
+  </si>
+  <si>
+    <t>Palabras  que más se repiten en las direcciones</t>
+  </si>
+  <si>
+    <t>MALL JARDIN</t>
+  </si>
+  <si>
+    <t>SAN MARINO</t>
   </si>
 </sst>
 </file>
@@ -446,12 +485,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55ECB879-B025-431C-B1DF-B099AB1BBF27}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="27.77734375" customWidth="1"/>
-    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="41" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -539,7 +578,65 @@
         <v>6</v>
       </c>
     </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>